<commit_message>
fix(cli): correct iodine fixture header
</commit_message>
<xml_diff>
--- a/apps/cli/tests/fixtures/food/mext_table_fixture.xlsx
+++ b/apps/cli/tests/fixtures/food/mext_table_fixture.xlsx
@@ -480,7 +480,7 @@
           <t>炭水化物</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>無 機 質</t>
         </is>
@@ -511,6 +511,11 @@
       <c r="M4" t="inlineStr">
         <is>
           <t>食物繊維総量</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ヨウ素</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">

</xml_diff>

<commit_message>
test(cli): align duplicate food fixture groups
</commit_message>
<xml_diff>
--- a/apps/cli/tests/fixtures/food/mext_table_fixture.xlsx
+++ b/apps/cli/tests/fixtures/food/mext_table_fixture.xlsx
@@ -1005,7 +1005,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1064,7 +1064,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">

</xml_diff>